<commit_message>
Chunk 11 progress 05:21 UTC
</commit_message>
<xml_diff>
--- a/gsmarena_new_2026-06-03.xlsx
+++ b/gsmarena_new_2026-06-03.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DK88"/>
+  <dimension ref="A1:DK90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22566,55 +22566,37 @@
           <t>2018, April. Released 2018, April</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>2018</t>
-        </is>
+      <c r="H67" t="n">
+        <v>2018</v>
       </c>
       <c r="I67" t="inlineStr">
         <is>
           <t>Discontinued</t>
         </is>
       </c>
-      <c r="J67" t="inlineStr">
-        <is>
-          <t>163</t>
-        </is>
-      </c>
-      <c r="K67" t="inlineStr">
-        <is>
-          <t>76.6</t>
-        </is>
-      </c>
-      <c r="L67" t="inlineStr">
-        <is>
-          <t>13.9</t>
-        </is>
-      </c>
-      <c r="M67" t="inlineStr">
-        <is>
-          <t>256</t>
-        </is>
-      </c>
-      <c r="N67" t="inlineStr">
-        <is>
-          <t>5.5</t>
-        </is>
-      </c>
-      <c r="O67" t="inlineStr">
-        <is>
-          <t>720</t>
-        </is>
-      </c>
-      <c r="P67" t="inlineStr">
-        <is>
-          <t>1440</t>
-        </is>
-      </c>
-      <c r="Q67" t="inlineStr">
-        <is>
-          <t>293</t>
-        </is>
+      <c r="J67" t="n">
+        <v>163</v>
+      </c>
+      <c r="K67" t="n">
+        <v>76.59999999999999</v>
+      </c>
+      <c r="L67" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="M67" t="n">
+        <v>256</v>
+      </c>
+      <c r="N67" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="O67" t="n">
+        <v>720</v>
+      </c>
+      <c r="P67" t="n">
+        <v>1440</v>
+      </c>
+      <c r="Q67" t="n">
+        <v>293</v>
       </c>
       <c r="R67" t="inlineStr">
         <is>
@@ -22626,20 +22608,14 @@
           <t>2GB</t>
         </is>
       </c>
-      <c r="T67" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="U67" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="V67" t="inlineStr">
-        <is>
-          <t>5500</t>
-        </is>
+      <c r="T67" t="n">
+        <v>8</v>
+      </c>
+      <c r="U67" t="n">
+        <v>5</v>
+      </c>
+      <c r="V67" t="n">
+        <v>5500</v>
       </c>
       <c r="W67" t="inlineStr"/>
       <c r="X67" t="inlineStr"/>
@@ -22919,55 +22895,37 @@
           <t>2014, September. Released 2014, September</t>
         </is>
       </c>
-      <c r="H68" t="inlineStr">
-        <is>
-          <t>2014</t>
-        </is>
+      <c r="H68" t="n">
+        <v>2014</v>
       </c>
       <c r="I68" t="inlineStr">
         <is>
           <t>Discontinued</t>
         </is>
       </c>
-      <c r="J68" t="inlineStr">
-        <is>
-          <t>148</t>
-        </is>
-      </c>
-      <c r="K68" t="inlineStr">
-        <is>
-          <t>74</t>
-        </is>
-      </c>
-      <c r="L68" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="M68" t="inlineStr">
-        <is>
-          <t>180</t>
-        </is>
-      </c>
-      <c r="N68" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="O68" t="inlineStr">
-        <is>
-          <t>720</t>
-        </is>
-      </c>
-      <c r="P68" t="inlineStr">
-        <is>
-          <t>1280</t>
-        </is>
-      </c>
-      <c r="Q68" t="inlineStr">
-        <is>
-          <t>294</t>
-        </is>
+      <c r="J68" t="n">
+        <v>148</v>
+      </c>
+      <c r="K68" t="n">
+        <v>74</v>
+      </c>
+      <c r="L68" t="n">
+        <v>9</v>
+      </c>
+      <c r="M68" t="n">
+        <v>180</v>
+      </c>
+      <c r="N68" t="n">
+        <v>5</v>
+      </c>
+      <c r="O68" t="n">
+        <v>720</v>
+      </c>
+      <c r="P68" t="n">
+        <v>1280</v>
+      </c>
+      <c r="Q68" t="n">
+        <v>294</v>
       </c>
       <c r="R68" t="inlineStr">
         <is>
@@ -22979,16 +22937,12 @@
           <t>512MB</t>
         </is>
       </c>
-      <c r="T68" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
+      <c r="T68" t="n">
+        <v>8</v>
       </c>
       <c r="U68" t="inlineStr"/>
-      <c r="V68" t="inlineStr">
-        <is>
-          <t>2000</t>
-        </is>
+      <c r="V68" t="n">
+        <v>2000</v>
       </c>
       <c r="W68" t="inlineStr"/>
       <c r="X68" t="inlineStr"/>
@@ -23252,55 +23206,37 @@
           <t>2014, June. Released 2014, June</t>
         </is>
       </c>
-      <c r="H69" t="inlineStr">
-        <is>
-          <t>2014</t>
-        </is>
+      <c r="H69" t="n">
+        <v>2014</v>
       </c>
       <c r="I69" t="inlineStr">
         <is>
           <t>Discontinued</t>
         </is>
       </c>
-      <c r="J69" t="inlineStr">
-        <is>
-          <t>125.5</t>
-        </is>
-      </c>
-      <c r="K69" t="inlineStr">
-        <is>
-          <t>65</t>
-        </is>
-      </c>
-      <c r="L69" t="inlineStr">
-        <is>
-          <t>9.4</t>
-        </is>
-      </c>
-      <c r="M69" t="inlineStr">
-        <is>
-          <t>110</t>
-        </is>
-      </c>
-      <c r="N69" t="inlineStr">
-        <is>
-          <t>4.0</t>
-        </is>
-      </c>
-      <c r="O69" t="inlineStr">
-        <is>
-          <t>480</t>
-        </is>
-      </c>
-      <c r="P69" t="inlineStr">
-        <is>
-          <t>800</t>
-        </is>
-      </c>
-      <c r="Q69" t="inlineStr">
-        <is>
-          <t>233</t>
-        </is>
+      <c r="J69" t="n">
+        <v>125.5</v>
+      </c>
+      <c r="K69" t="n">
+        <v>65</v>
+      </c>
+      <c r="L69" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="M69" t="n">
+        <v>110</v>
+      </c>
+      <c r="N69" t="n">
+        <v>4</v>
+      </c>
+      <c r="O69" t="n">
+        <v>480</v>
+      </c>
+      <c r="P69" t="n">
+        <v>800</v>
+      </c>
+      <c r="Q69" t="n">
+        <v>233</v>
       </c>
       <c r="R69" t="inlineStr">
         <is>
@@ -23312,16 +23248,12 @@
           <t>512MB</t>
         </is>
       </c>
-      <c r="T69" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
+      <c r="T69" t="n">
+        <v>8</v>
       </c>
       <c r="U69" t="inlineStr"/>
-      <c r="V69" t="inlineStr">
-        <is>
-          <t>1500</t>
-        </is>
+      <c r="V69" t="n">
+        <v>1500</v>
       </c>
       <c r="W69" t="inlineStr"/>
       <c r="X69" t="inlineStr"/>
@@ -23581,55 +23513,37 @@
           <t>2014, June. Released 2014, June</t>
         </is>
       </c>
-      <c r="H70" t="inlineStr">
-        <is>
-          <t>2014</t>
-        </is>
+      <c r="H70" t="n">
+        <v>2014</v>
       </c>
       <c r="I70" t="inlineStr">
         <is>
           <t>Discontinued</t>
         </is>
       </c>
-      <c r="J70" t="inlineStr">
-        <is>
-          <t>116</t>
-        </is>
-      </c>
-      <c r="K70" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="L70" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="M70" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="N70" t="inlineStr">
-        <is>
-          <t>3.5</t>
-        </is>
-      </c>
-      <c r="O70" t="inlineStr">
-        <is>
-          <t>320</t>
-        </is>
-      </c>
-      <c r="P70" t="inlineStr">
-        <is>
-          <t>480</t>
-        </is>
-      </c>
-      <c r="Q70" t="inlineStr">
-        <is>
-          <t>165</t>
-        </is>
+      <c r="J70" t="n">
+        <v>116</v>
+      </c>
+      <c r="K70" t="n">
+        <v>61</v>
+      </c>
+      <c r="L70" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="M70" t="n">
+        <v>100</v>
+      </c>
+      <c r="N70" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="O70" t="n">
+        <v>320</v>
+      </c>
+      <c r="P70" t="n">
+        <v>480</v>
+      </c>
+      <c r="Q70" t="n">
+        <v>165</v>
       </c>
       <c r="R70" t="inlineStr">
         <is>
@@ -23641,16 +23555,12 @@
           <t>256MB</t>
         </is>
       </c>
-      <c r="T70" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
+      <c r="T70" t="n">
+        <v>15</v>
       </c>
       <c r="U70" t="inlineStr"/>
-      <c r="V70" t="inlineStr">
-        <is>
-          <t>1200</t>
-        </is>
+      <c r="V70" t="n">
+        <v>1200</v>
       </c>
       <c r="W70" t="inlineStr"/>
       <c r="X70" t="inlineStr"/>
@@ -23902,55 +23812,37 @@
           <t>2015, January. Released 2015, January</t>
         </is>
       </c>
-      <c r="H71" t="inlineStr">
-        <is>
-          <t>2015</t>
-        </is>
+      <c r="H71" t="n">
+        <v>2015</v>
       </c>
       <c r="I71" t="inlineStr">
         <is>
           <t>Discontinued</t>
         </is>
       </c>
-      <c r="J71" t="inlineStr">
-        <is>
-          <t>127.5</t>
-        </is>
-      </c>
-      <c r="K71" t="inlineStr">
-        <is>
-          <t>64.9</t>
-        </is>
-      </c>
-      <c r="L71" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="M71" t="inlineStr">
-        <is>
-          <t>128</t>
-        </is>
-      </c>
-      <c r="N71" t="inlineStr">
-        <is>
-          <t>4.0</t>
-        </is>
-      </c>
-      <c r="O71" t="inlineStr">
-        <is>
-          <t>480</t>
-        </is>
-      </c>
-      <c r="P71" t="inlineStr">
-        <is>
-          <t>800</t>
-        </is>
-      </c>
-      <c r="Q71" t="inlineStr">
-        <is>
-          <t>233</t>
-        </is>
+      <c r="J71" t="n">
+        <v>127.5</v>
+      </c>
+      <c r="K71" t="n">
+        <v>64.90000000000001</v>
+      </c>
+      <c r="L71" t="n">
+        <v>11</v>
+      </c>
+      <c r="M71" t="n">
+        <v>128</v>
+      </c>
+      <c r="N71" t="n">
+        <v>4</v>
+      </c>
+      <c r="O71" t="n">
+        <v>480</v>
+      </c>
+      <c r="P71" t="n">
+        <v>800</v>
+      </c>
+      <c r="Q71" t="n">
+        <v>233</v>
       </c>
       <c r="R71" t="inlineStr">
         <is>
@@ -23962,32 +23854,22 @@
           <t>512MB</t>
         </is>
       </c>
-      <c r="T71" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="U71" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="V71" t="inlineStr">
-        <is>
-          <t>1400</t>
-        </is>
+      <c r="T71" t="n">
+        <v>8</v>
+      </c>
+      <c r="U71" t="n">
+        <v>3</v>
+      </c>
+      <c r="V71" t="n">
+        <v>1400</v>
       </c>
       <c r="W71" t="inlineStr"/>
       <c r="X71" t="inlineStr"/>
-      <c r="Y71" t="inlineStr">
-        <is>
-          <t>0.66</t>
-        </is>
-      </c>
-      <c r="Z71" t="inlineStr">
-        <is>
-          <t>1.38</t>
-        </is>
+      <c r="Y71" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="Z71" t="n">
+        <v>1.38</v>
       </c>
       <c r="AA71" t="inlineStr"/>
       <c r="AB71" t="inlineStr"/>
@@ -24263,55 +24145,37 @@
           <t>2015, January. Released 2015, January</t>
         </is>
       </c>
-      <c r="H72" t="inlineStr">
-        <is>
-          <t>2015</t>
-        </is>
+      <c r="H72" t="n">
+        <v>2015</v>
       </c>
       <c r="I72" t="inlineStr">
         <is>
           <t>Discontinued</t>
         </is>
       </c>
-      <c r="J72" t="inlineStr">
-        <is>
-          <t>122</t>
-        </is>
-      </c>
-      <c r="K72" t="inlineStr">
-        <is>
-          <t>63</t>
-        </is>
-      </c>
-      <c r="L72" t="inlineStr">
-        <is>
-          <t>10.7</t>
-        </is>
-      </c>
-      <c r="M72" t="inlineStr">
-        <is>
-          <t>112</t>
-        </is>
-      </c>
-      <c r="N72" t="inlineStr">
-        <is>
-          <t>4.0</t>
-        </is>
-      </c>
-      <c r="O72" t="inlineStr">
-        <is>
-          <t>480</t>
-        </is>
-      </c>
-      <c r="P72" t="inlineStr">
-        <is>
-          <t>800</t>
-        </is>
-      </c>
-      <c r="Q72" t="inlineStr">
-        <is>
-          <t>233</t>
-        </is>
+      <c r="J72" t="n">
+        <v>122</v>
+      </c>
+      <c r="K72" t="n">
+        <v>63</v>
+      </c>
+      <c r="L72" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="M72" t="n">
+        <v>112</v>
+      </c>
+      <c r="N72" t="n">
+        <v>4</v>
+      </c>
+      <c r="O72" t="n">
+        <v>480</v>
+      </c>
+      <c r="P72" t="n">
+        <v>800</v>
+      </c>
+      <c r="Q72" t="n">
+        <v>233</v>
       </c>
       <c r="R72" t="inlineStr">
         <is>
@@ -24323,32 +24187,22 @@
           <t>256MB</t>
         </is>
       </c>
-      <c r="T72" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="U72" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="V72" t="inlineStr">
-        <is>
-          <t>1450</t>
-        </is>
+      <c r="T72" t="n">
+        <v>5</v>
+      </c>
+      <c r="U72" t="n">
+        <v>3</v>
+      </c>
+      <c r="V72" t="n">
+        <v>1450</v>
       </c>
       <c r="W72" t="inlineStr"/>
       <c r="X72" t="inlineStr"/>
-      <c r="Y72" t="inlineStr">
-        <is>
-          <t>0.49</t>
-        </is>
-      </c>
-      <c r="Z72" t="inlineStr">
-        <is>
-          <t>0.74</t>
-        </is>
+      <c r="Y72" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="Z72" t="n">
+        <v>0.74</v>
       </c>
       <c r="AA72" t="inlineStr"/>
       <c r="AB72" t="inlineStr"/>
@@ -24624,55 +24478,37 @@
           <t>2014, November. Released 2014, November</t>
         </is>
       </c>
-      <c r="H73" t="inlineStr">
-        <is>
-          <t>2014</t>
-        </is>
+      <c r="H73" t="n">
+        <v>2014</v>
       </c>
       <c r="I73" t="inlineStr">
         <is>
           <t>Discontinued</t>
         </is>
       </c>
-      <c r="J73" t="inlineStr">
-        <is>
-          <t>113.4</t>
-        </is>
-      </c>
-      <c r="K73" t="inlineStr">
-        <is>
-          <t>60.2</t>
-        </is>
-      </c>
-      <c r="L73" t="inlineStr">
-        <is>
-          <t>12.5</t>
-        </is>
-      </c>
-      <c r="M73" t="inlineStr">
-        <is>
-          <t>88.5</t>
-        </is>
-      </c>
-      <c r="N73" t="inlineStr">
-        <is>
-          <t>3.5</t>
-        </is>
-      </c>
-      <c r="O73" t="inlineStr">
-        <is>
-          <t>320</t>
-        </is>
-      </c>
-      <c r="P73" t="inlineStr">
-        <is>
-          <t>480</t>
-        </is>
-      </c>
-      <c r="Q73" t="inlineStr">
-        <is>
-          <t>165</t>
-        </is>
+      <c r="J73" t="n">
+        <v>113.4</v>
+      </c>
+      <c r="K73" t="n">
+        <v>60.2</v>
+      </c>
+      <c r="L73" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="M73" t="n">
+        <v>88.5</v>
+      </c>
+      <c r="N73" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="O73" t="n">
+        <v>320</v>
+      </c>
+      <c r="P73" t="n">
+        <v>480</v>
+      </c>
+      <c r="Q73" t="n">
+        <v>165</v>
       </c>
       <c r="R73" t="inlineStr">
         <is>
@@ -24684,16 +24520,12 @@
           <t>256MB</t>
         </is>
       </c>
-      <c r="T73" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="T73" t="n">
+        <v>2</v>
       </c>
       <c r="U73" t="inlineStr"/>
-      <c r="V73" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
+      <c r="V73" t="n">
+        <v>1000</v>
       </c>
       <c r="W73" t="inlineStr"/>
       <c r="X73" t="inlineStr"/>
@@ -24961,55 +24793,37 @@
           <t>2014, September. Released 2014, October</t>
         </is>
       </c>
-      <c r="H74" t="inlineStr">
-        <is>
-          <t>2014</t>
-        </is>
+      <c r="H74" t="n">
+        <v>2014</v>
       </c>
       <c r="I74" t="inlineStr">
         <is>
           <t>Discontinued</t>
         </is>
       </c>
-      <c r="J74" t="inlineStr">
-        <is>
-          <t>111.4</t>
-        </is>
-      </c>
-      <c r="K74" t="inlineStr">
-        <is>
-          <t>51.5</t>
-        </is>
-      </c>
-      <c r="L74" t="inlineStr">
-        <is>
-          <t>15.6</t>
-        </is>
-      </c>
-      <c r="M74" t="inlineStr">
-        <is>
-          <t>110</t>
-        </is>
-      </c>
-      <c r="N74" t="inlineStr">
-        <is>
-          <t>2.2</t>
-        </is>
-      </c>
-      <c r="O74" t="inlineStr">
-        <is>
-          <t>176</t>
-        </is>
-      </c>
-      <c r="P74" t="inlineStr">
-        <is>
-          <t>220</t>
-        </is>
-      </c>
-      <c r="Q74" t="inlineStr">
-        <is>
-          <t>128</t>
-        </is>
+      <c r="J74" t="n">
+        <v>111.4</v>
+      </c>
+      <c r="K74" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="L74" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="M74" t="n">
+        <v>110</v>
+      </c>
+      <c r="N74" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="O74" t="n">
+        <v>176</v>
+      </c>
+      <c r="P74" t="n">
+        <v>220</v>
+      </c>
+      <c r="Q74" t="n">
+        <v>128</v>
       </c>
       <c r="R74" t="inlineStr">
         <is>
@@ -25021,26 +24835,18 @@
           <t>32MB</t>
         </is>
       </c>
-      <c r="T74" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="T74" t="n">
+        <v>2</v>
       </c>
       <c r="U74" t="inlineStr"/>
-      <c r="V74" t="inlineStr">
-        <is>
-          <t>900</t>
-        </is>
-      </c>
-      <c r="W74" t="inlineStr">
-        <is>
-          <t>1.33</t>
-        </is>
-      </c>
-      <c r="X74" t="inlineStr">
-        <is>
-          <t>1.28</t>
-        </is>
+      <c r="V74" t="n">
+        <v>900</v>
+      </c>
+      <c r="W74" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="X74" t="n">
+        <v>1.28</v>
       </c>
       <c r="Y74" t="inlineStr"/>
       <c r="Z74" t="inlineStr"/>
@@ -25330,55 +25136,37 @@
           <t>2014, October. Released 2014, October</t>
         </is>
       </c>
-      <c r="H75" t="inlineStr">
-        <is>
-          <t>2014</t>
-        </is>
+      <c r="H75" t="n">
+        <v>2014</v>
       </c>
       <c r="I75" t="inlineStr">
         <is>
           <t>Discontinued</t>
         </is>
       </c>
-      <c r="J75" t="inlineStr">
-        <is>
-          <t>150.4</t>
-        </is>
-      </c>
-      <c r="K75" t="inlineStr">
-        <is>
-          <t>77.2</t>
-        </is>
-      </c>
-      <c r="L75" t="inlineStr">
-        <is>
-          <t>8.5</t>
-        </is>
-      </c>
-      <c r="M75" t="inlineStr">
-        <is>
-          <t>157</t>
-        </is>
-      </c>
-      <c r="N75" t="inlineStr">
-        <is>
-          <t>5.5</t>
-        </is>
-      </c>
-      <c r="O75" t="inlineStr">
-        <is>
-          <t>540</t>
-        </is>
-      </c>
-      <c r="P75" t="inlineStr">
-        <is>
-          <t>960</t>
-        </is>
-      </c>
-      <c r="Q75" t="inlineStr">
-        <is>
-          <t>200</t>
-        </is>
+      <c r="J75" t="n">
+        <v>150.4</v>
+      </c>
+      <c r="K75" t="n">
+        <v>77.2</v>
+      </c>
+      <c r="L75" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="M75" t="n">
+        <v>157</v>
+      </c>
+      <c r="N75" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="O75" t="n">
+        <v>540</v>
+      </c>
+      <c r="P75" t="n">
+        <v>960</v>
+      </c>
+      <c r="Q75" t="n">
+        <v>200</v>
       </c>
       <c r="R75" t="inlineStr">
         <is>
@@ -25390,20 +25178,14 @@
           <t>1GB</t>
         </is>
       </c>
-      <c r="T75" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="U75" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="V75" t="inlineStr">
-        <is>
-          <t>2300</t>
-        </is>
+      <c r="T75" t="n">
+        <v>8</v>
+      </c>
+      <c r="U75" t="n">
+        <v>2</v>
+      </c>
+      <c r="V75" t="n">
+        <v>2300</v>
       </c>
       <c r="W75" t="inlineStr"/>
       <c r="X75" t="inlineStr"/>
@@ -25671,58 +25453,40 @@
           <t>2012, Q1</t>
         </is>
       </c>
-      <c r="H76" t="inlineStr">
-        <is>
-          <t>2012</t>
-        </is>
+      <c r="H76" t="n">
+        <v>2012</v>
       </c>
       <c r="I76" t="inlineStr">
         <is>
           <t>Discontinued</t>
         </is>
       </c>
-      <c r="J76" t="inlineStr">
-        <is>
-          <t>118</t>
-        </is>
-      </c>
-      <c r="K76" t="inlineStr">
-        <is>
-          <t>49.8</t>
-        </is>
-      </c>
-      <c r="L76" t="inlineStr">
-        <is>
-          <t>13.5</t>
-        </is>
-      </c>
-      <c r="M76" t="inlineStr">
-        <is>
-          <t>79</t>
-        </is>
-      </c>
-      <c r="N76" t="inlineStr">
-        <is>
-          <t>2.0</t>
-        </is>
-      </c>
-      <c r="O76" t="inlineStr">
-        <is>
-          <t>176</t>
-        </is>
-      </c>
-      <c r="P76" t="inlineStr">
-        <is>
-          <t>220</t>
-        </is>
+      <c r="J76" t="n">
+        <v>118</v>
+      </c>
+      <c r="K76" t="n">
+        <v>49.8</v>
+      </c>
+      <c r="L76" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="M76" t="n">
+        <v>79</v>
+      </c>
+      <c r="N76" t="n">
+        <v>2</v>
+      </c>
+      <c r="O76" t="n">
+        <v>176</v>
+      </c>
+      <c r="P76" t="n">
+        <v>220</v>
       </c>
       <c r="Q76" t="inlineStr"/>
       <c r="R76" t="inlineStr"/>
       <c r="S76" t="inlineStr"/>
-      <c r="T76" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="T76" t="n">
+        <v>3</v>
       </c>
       <c r="U76" t="inlineStr"/>
       <c r="V76" t="inlineStr"/>
@@ -25992,50 +25756,34 @@
           <t>2012, January. Released 2012, January</t>
         </is>
       </c>
-      <c r="H77" t="inlineStr">
-        <is>
-          <t>2012</t>
-        </is>
+      <c r="H77" t="n">
+        <v>2012</v>
       </c>
       <c r="I77" t="inlineStr">
         <is>
           <t>Discontinued</t>
         </is>
       </c>
-      <c r="J77" t="inlineStr">
-        <is>
-          <t>107</t>
-        </is>
-      </c>
-      <c r="K77" t="inlineStr">
-        <is>
-          <t>45</t>
-        </is>
-      </c>
-      <c r="L77" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="M77" t="inlineStr">
-        <is>
-          <t>63</t>
-        </is>
-      </c>
-      <c r="N77" t="inlineStr">
-        <is>
-          <t>1.8</t>
-        </is>
-      </c>
-      <c r="O77" t="inlineStr">
-        <is>
-          <t>160</t>
-        </is>
-      </c>
-      <c r="P77" t="inlineStr">
-        <is>
-          <t>240</t>
-        </is>
+      <c r="J77" t="n">
+        <v>107</v>
+      </c>
+      <c r="K77" t="n">
+        <v>45</v>
+      </c>
+      <c r="L77" t="n">
+        <v>12</v>
+      </c>
+      <c r="M77" t="n">
+        <v>63</v>
+      </c>
+      <c r="N77" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="O77" t="n">
+        <v>160</v>
+      </c>
+      <c r="P77" t="n">
+        <v>240</v>
       </c>
       <c r="Q77" t="inlineStr"/>
       <c r="R77" t="inlineStr"/>
@@ -26305,62 +26053,42 @@
           <t>2011, Q4. Released 2011, December</t>
         </is>
       </c>
-      <c r="H78" t="inlineStr">
-        <is>
-          <t>2011</t>
-        </is>
+      <c r="H78" t="n">
+        <v>2011</v>
       </c>
       <c r="I78" t="inlineStr">
         <is>
           <t>Discontinued</t>
         </is>
       </c>
-      <c r="J78" t="inlineStr">
-        <is>
-          <t>105.5</t>
-        </is>
-      </c>
-      <c r="K78" t="inlineStr">
-        <is>
-          <t>58</t>
-        </is>
-      </c>
-      <c r="L78" t="inlineStr">
-        <is>
-          <t>11.7</t>
-        </is>
-      </c>
-      <c r="M78" t="inlineStr">
-        <is>
-          <t>90</t>
-        </is>
-      </c>
-      <c r="N78" t="inlineStr">
-        <is>
-          <t>2.4</t>
-        </is>
-      </c>
-      <c r="O78" t="inlineStr">
-        <is>
-          <t>320</t>
-        </is>
-      </c>
-      <c r="P78" t="inlineStr">
-        <is>
-          <t>240</t>
-        </is>
-      </c>
-      <c r="Q78" t="inlineStr">
-        <is>
-          <t>167</t>
-        </is>
+      <c r="J78" t="n">
+        <v>105.5</v>
+      </c>
+      <c r="K78" t="n">
+        <v>58</v>
+      </c>
+      <c r="L78" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="M78" t="n">
+        <v>90</v>
+      </c>
+      <c r="N78" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="O78" t="n">
+        <v>320</v>
+      </c>
+      <c r="P78" t="n">
+        <v>240</v>
+      </c>
+      <c r="Q78" t="n">
+        <v>167</v>
       </c>
       <c r="R78" t="inlineStr"/>
       <c r="S78" t="inlineStr"/>
-      <c r="T78" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="T78" t="n">
+        <v>2</v>
       </c>
       <c r="U78" t="inlineStr"/>
       <c r="V78" t="inlineStr"/>
@@ -26626,58 +26354,40 @@
           <t>2011. Released 2011</t>
         </is>
       </c>
-      <c r="H79" t="inlineStr">
-        <is>
-          <t>2011</t>
-        </is>
+      <c r="H79" t="n">
+        <v>2011</v>
       </c>
       <c r="I79" t="inlineStr">
         <is>
           <t>Discontinued</t>
         </is>
       </c>
-      <c r="J79" t="inlineStr">
-        <is>
-          <t>111</t>
-        </is>
-      </c>
-      <c r="K79" t="inlineStr">
-        <is>
-          <t>51.5</t>
-        </is>
-      </c>
-      <c r="L79" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="M79" t="inlineStr">
-        <is>
-          <t>110</t>
-        </is>
-      </c>
-      <c r="N79" t="inlineStr">
-        <is>
-          <t>2.2</t>
-        </is>
-      </c>
-      <c r="O79" t="inlineStr">
-        <is>
-          <t>176</t>
-        </is>
-      </c>
-      <c r="P79" t="inlineStr">
-        <is>
-          <t>220</t>
-        </is>
+      <c r="J79" t="n">
+        <v>111</v>
+      </c>
+      <c r="K79" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="L79" t="n">
+        <v>15</v>
+      </c>
+      <c r="M79" t="n">
+        <v>110</v>
+      </c>
+      <c r="N79" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="O79" t="n">
+        <v>176</v>
+      </c>
+      <c r="P79" t="n">
+        <v>220</v>
       </c>
       <c r="Q79" t="inlineStr"/>
       <c r="R79" t="inlineStr"/>
       <c r="S79" t="inlineStr"/>
-      <c r="T79" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="T79" t="n">
+        <v>3</v>
       </c>
       <c r="U79" t="inlineStr"/>
       <c r="V79" t="inlineStr"/>
@@ -26927,55 +26637,37 @@
           <t>2011, Q3</t>
         </is>
       </c>
-      <c r="H80" t="inlineStr">
-        <is>
-          <t>2011</t>
-        </is>
+      <c r="H80" t="n">
+        <v>2011</v>
       </c>
       <c r="I80" t="inlineStr">
         <is>
           <t>Discontinued</t>
         </is>
       </c>
-      <c r="J80" t="inlineStr">
-        <is>
-          <t>115.8</t>
-        </is>
-      </c>
-      <c r="K80" t="inlineStr">
-        <is>
-          <t>62</t>
-        </is>
-      </c>
-      <c r="L80" t="inlineStr">
-        <is>
-          <t>13.2</t>
-        </is>
-      </c>
-      <c r="M80" t="inlineStr">
-        <is>
-          <t>110</t>
-        </is>
-      </c>
-      <c r="N80" t="inlineStr">
-        <is>
-          <t>2.3</t>
-        </is>
-      </c>
-      <c r="O80" t="inlineStr">
-        <is>
-          <t>320</t>
-        </is>
-      </c>
-      <c r="P80" t="inlineStr">
-        <is>
-          <t>240</t>
-        </is>
-      </c>
-      <c r="Q80" t="inlineStr">
-        <is>
-          <t>174</t>
-        </is>
+      <c r="J80" t="n">
+        <v>115.8</v>
+      </c>
+      <c r="K80" t="n">
+        <v>62</v>
+      </c>
+      <c r="L80" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="M80" t="n">
+        <v>110</v>
+      </c>
+      <c r="N80" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="O80" t="n">
+        <v>320</v>
+      </c>
+      <c r="P80" t="n">
+        <v>240</v>
+      </c>
+      <c r="Q80" t="n">
+        <v>174</v>
       </c>
       <c r="R80" t="inlineStr">
         <is>
@@ -26983,10 +26675,8 @@
         </is>
       </c>
       <c r="S80" t="inlineStr"/>
-      <c r="T80" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="T80" t="n">
+        <v>2</v>
       </c>
       <c r="U80" t="inlineStr"/>
       <c r="V80" t="inlineStr"/>
@@ -27260,55 +26950,37 @@
           <t>2011, Q2</t>
         </is>
       </c>
-      <c r="H81" t="inlineStr">
-        <is>
-          <t>2011</t>
-        </is>
+      <c r="H81" t="n">
+        <v>2011</v>
       </c>
       <c r="I81" t="inlineStr">
         <is>
           <t>Discontinued</t>
         </is>
       </c>
-      <c r="J81" t="inlineStr">
-        <is>
-          <t>117</t>
-        </is>
-      </c>
-      <c r="K81" t="inlineStr">
-        <is>
-          <t>57</t>
-        </is>
-      </c>
-      <c r="L81" t="inlineStr">
-        <is>
-          <t>12.1</t>
-        </is>
-      </c>
-      <c r="M81" t="inlineStr">
-        <is>
-          <t>106</t>
-        </is>
-      </c>
-      <c r="N81" t="inlineStr">
-        <is>
-          <t>3.2</t>
-        </is>
-      </c>
-      <c r="O81" t="inlineStr">
-        <is>
-          <t>240</t>
-        </is>
-      </c>
-      <c r="P81" t="inlineStr">
-        <is>
-          <t>400</t>
-        </is>
-      </c>
-      <c r="Q81" t="inlineStr">
-        <is>
-          <t>146</t>
-        </is>
+      <c r="J81" t="n">
+        <v>117</v>
+      </c>
+      <c r="K81" t="n">
+        <v>57</v>
+      </c>
+      <c r="L81" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="M81" t="n">
+        <v>106</v>
+      </c>
+      <c r="N81" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="O81" t="n">
+        <v>240</v>
+      </c>
+      <c r="P81" t="n">
+        <v>400</v>
+      </c>
+      <c r="Q81" t="n">
+        <v>146</v>
       </c>
       <c r="R81" t="inlineStr">
         <is>
@@ -27316,16 +26988,12 @@
         </is>
       </c>
       <c r="S81" t="inlineStr"/>
-      <c r="T81" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="T81" t="n">
+        <v>2</v>
       </c>
       <c r="U81" t="inlineStr"/>
-      <c r="V81" t="inlineStr">
-        <is>
-          <t>1100</t>
-        </is>
+      <c r="V81" t="n">
+        <v>1100</v>
       </c>
       <c r="W81" t="inlineStr"/>
       <c r="X81" t="inlineStr"/>
@@ -27581,55 +27249,37 @@
           <t>2011, Q2</t>
         </is>
       </c>
-      <c r="H82" t="inlineStr">
-        <is>
-          <t>2011</t>
-        </is>
+      <c r="H82" t="n">
+        <v>2011</v>
       </c>
       <c r="I82" t="inlineStr">
         <is>
           <t>Discontinued</t>
         </is>
       </c>
-      <c r="J82" t="inlineStr">
-        <is>
-          <t>107</t>
-        </is>
-      </c>
-      <c r="K82" t="inlineStr">
-        <is>
-          <t>57</t>
-        </is>
-      </c>
-      <c r="L82" t="inlineStr">
-        <is>
-          <t>11.8</t>
-        </is>
-      </c>
-      <c r="M82" t="inlineStr">
-        <is>
-          <t>106</t>
-        </is>
-      </c>
-      <c r="N82" t="inlineStr">
-        <is>
-          <t>3.0</t>
-        </is>
-      </c>
-      <c r="O82" t="inlineStr">
-        <is>
-          <t>240</t>
-        </is>
-      </c>
-      <c r="P82" t="inlineStr">
-        <is>
-          <t>320</t>
-        </is>
-      </c>
-      <c r="Q82" t="inlineStr">
-        <is>
-          <t>133</t>
-        </is>
+      <c r="J82" t="n">
+        <v>107</v>
+      </c>
+      <c r="K82" t="n">
+        <v>57</v>
+      </c>
+      <c r="L82" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="M82" t="n">
+        <v>106</v>
+      </c>
+      <c r="N82" t="n">
+        <v>3</v>
+      </c>
+      <c r="O82" t="n">
+        <v>240</v>
+      </c>
+      <c r="P82" t="n">
+        <v>320</v>
+      </c>
+      <c r="Q82" t="n">
+        <v>133</v>
       </c>
       <c r="R82" t="inlineStr">
         <is>
@@ -27637,16 +27287,12 @@
         </is>
       </c>
       <c r="S82" t="inlineStr"/>
-      <c r="T82" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="T82" t="n">
+        <v>2</v>
       </c>
       <c r="U82" t="inlineStr"/>
-      <c r="V82" t="inlineStr">
-        <is>
-          <t>700</t>
-        </is>
+      <c r="V82" t="n">
+        <v>700</v>
       </c>
       <c r="W82" t="inlineStr"/>
       <c r="X82" t="inlineStr"/>
@@ -27898,46 +27544,32 @@
           <t>2011. Released 2011</t>
         </is>
       </c>
-      <c r="H83" t="inlineStr">
-        <is>
-          <t>2011</t>
-        </is>
+      <c r="H83" t="n">
+        <v>2011</v>
       </c>
       <c r="I83" t="inlineStr">
         <is>
           <t>Discontinued</t>
         </is>
       </c>
-      <c r="J83" t="inlineStr">
-        <is>
-          <t>103</t>
-        </is>
-      </c>
-      <c r="K83" t="inlineStr">
-        <is>
-          <t>56</t>
-        </is>
-      </c>
-      <c r="L83" t="inlineStr">
-        <is>
-          <t>13.5</t>
-        </is>
+      <c r="J83" t="n">
+        <v>103</v>
+      </c>
+      <c r="K83" t="n">
+        <v>56</v>
+      </c>
+      <c r="L83" t="n">
+        <v>13.5</v>
       </c>
       <c r="M83" t="inlineStr"/>
-      <c r="N83" t="inlineStr">
-        <is>
-          <t>2.0</t>
-        </is>
-      </c>
-      <c r="O83" t="inlineStr">
-        <is>
-          <t>240</t>
-        </is>
-      </c>
-      <c r="P83" t="inlineStr">
-        <is>
-          <t>320</t>
-        </is>
+      <c r="N83" t="n">
+        <v>2</v>
+      </c>
+      <c r="O83" t="n">
+        <v>240</v>
+      </c>
+      <c r="P83" t="n">
+        <v>320</v>
       </c>
       <c r="Q83" t="inlineStr"/>
       <c r="R83" t="inlineStr"/>
@@ -28195,55 +27827,37 @@
           <t>2011. Released 2011</t>
         </is>
       </c>
-      <c r="H84" t="inlineStr">
-        <is>
-          <t>2011</t>
-        </is>
+      <c r="H84" t="n">
+        <v>2011</v>
       </c>
       <c r="I84" t="inlineStr">
         <is>
           <t>Discontinued</t>
         </is>
       </c>
-      <c r="J84" t="inlineStr">
-        <is>
-          <t>111</t>
-        </is>
-      </c>
-      <c r="K84" t="inlineStr">
-        <is>
-          <t>58.5</t>
-        </is>
-      </c>
-      <c r="L84" t="inlineStr">
-        <is>
-          <t>13.2</t>
-        </is>
-      </c>
-      <c r="M84" t="inlineStr">
-        <is>
-          <t>107</t>
-        </is>
-      </c>
-      <c r="N84" t="inlineStr">
-        <is>
-          <t>2.8</t>
-        </is>
-      </c>
-      <c r="O84" t="inlineStr">
-        <is>
-          <t>240</t>
-        </is>
-      </c>
-      <c r="P84" t="inlineStr">
-        <is>
-          <t>320</t>
-        </is>
-      </c>
-      <c r="Q84" t="inlineStr">
-        <is>
-          <t>143</t>
-        </is>
+      <c r="J84" t="n">
+        <v>111</v>
+      </c>
+      <c r="K84" t="n">
+        <v>58.5</v>
+      </c>
+      <c r="L84" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="M84" t="n">
+        <v>107</v>
+      </c>
+      <c r="N84" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="O84" t="n">
+        <v>240</v>
+      </c>
+      <c r="P84" t="n">
+        <v>320</v>
+      </c>
+      <c r="Q84" t="n">
+        <v>143</v>
       </c>
       <c r="R84" t="inlineStr">
         <is>
@@ -28251,10 +27865,8 @@
         </is>
       </c>
       <c r="S84" t="inlineStr"/>
-      <c r="T84" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
+      <c r="T84" t="n">
+        <v>15</v>
       </c>
       <c r="U84" t="inlineStr"/>
       <c r="V84" t="inlineStr"/>
@@ -28532,62 +28144,42 @@
           <t>2011. Released 2011</t>
         </is>
       </c>
-      <c r="H85" t="inlineStr">
-        <is>
-          <t>2011</t>
-        </is>
+      <c r="H85" t="n">
+        <v>2011</v>
       </c>
       <c r="I85" t="inlineStr">
         <is>
           <t>Discontinued</t>
         </is>
       </c>
-      <c r="J85" t="inlineStr">
-        <is>
-          <t>102</t>
-        </is>
-      </c>
-      <c r="K85" t="inlineStr">
-        <is>
-          <t>62</t>
-        </is>
-      </c>
-      <c r="L85" t="inlineStr">
-        <is>
-          <t>16.3</t>
-        </is>
-      </c>
-      <c r="M85" t="inlineStr">
-        <is>
-          <t>145</t>
-        </is>
-      </c>
-      <c r="N85" t="inlineStr">
-        <is>
-          <t>2.8</t>
-        </is>
-      </c>
-      <c r="O85" t="inlineStr">
-        <is>
-          <t>240</t>
-        </is>
-      </c>
-      <c r="P85" t="inlineStr">
-        <is>
-          <t>320</t>
-        </is>
-      </c>
-      <c r="Q85" t="inlineStr">
-        <is>
-          <t>143</t>
-        </is>
+      <c r="J85" t="n">
+        <v>102</v>
+      </c>
+      <c r="K85" t="n">
+        <v>62</v>
+      </c>
+      <c r="L85" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="M85" t="n">
+        <v>145</v>
+      </c>
+      <c r="N85" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="O85" t="n">
+        <v>240</v>
+      </c>
+      <c r="P85" t="n">
+        <v>320</v>
+      </c>
+      <c r="Q85" t="n">
+        <v>143</v>
       </c>
       <c r="R85" t="inlineStr"/>
       <c r="S85" t="inlineStr"/>
-      <c r="T85" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="T85" t="n">
+        <v>2</v>
       </c>
       <c r="U85" t="inlineStr"/>
       <c r="V85" t="inlineStr"/>
@@ -28853,50 +28445,34 @@
           <t>2011. Released 2011</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr">
-        <is>
-          <t>2011</t>
-        </is>
+      <c r="H86" t="n">
+        <v>2011</v>
       </c>
       <c r="I86" t="inlineStr">
         <is>
           <t>Discontinued</t>
         </is>
       </c>
-      <c r="J86" t="inlineStr">
-        <is>
-          <t>94</t>
-        </is>
-      </c>
-      <c r="K86" t="inlineStr">
-        <is>
-          <t>45</t>
-        </is>
-      </c>
-      <c r="L86" t="inlineStr">
-        <is>
-          <t>18.6</t>
-        </is>
-      </c>
-      <c r="M86" t="inlineStr">
-        <is>
-          <t>90</t>
-        </is>
-      </c>
-      <c r="N86" t="inlineStr">
-        <is>
-          <t>2.0</t>
-        </is>
-      </c>
-      <c r="O86" t="inlineStr">
-        <is>
-          <t>240</t>
-        </is>
-      </c>
-      <c r="P86" t="inlineStr">
-        <is>
-          <t>320</t>
-        </is>
+      <c r="J86" t="n">
+        <v>94</v>
+      </c>
+      <c r="K86" t="n">
+        <v>45</v>
+      </c>
+      <c r="L86" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="M86" t="n">
+        <v>90</v>
+      </c>
+      <c r="N86" t="n">
+        <v>2</v>
+      </c>
+      <c r="O86" t="n">
+        <v>240</v>
+      </c>
+      <c r="P86" t="n">
+        <v>320</v>
       </c>
       <c r="Q86" t="inlineStr"/>
       <c r="R86" t="inlineStr"/>
@@ -29158,55 +28734,37 @@
           <t>2011. Released 2011</t>
         </is>
       </c>
-      <c r="H87" t="inlineStr">
-        <is>
-          <t>2011</t>
-        </is>
+      <c r="H87" t="n">
+        <v>2011</v>
       </c>
       <c r="I87" t="inlineStr">
         <is>
           <t>Discontinued</t>
         </is>
       </c>
-      <c r="J87" t="inlineStr">
-        <is>
-          <t>118</t>
-        </is>
-      </c>
-      <c r="K87" t="inlineStr">
-        <is>
-          <t>53</t>
-        </is>
-      </c>
-      <c r="L87" t="inlineStr">
-        <is>
-          <t>15.8</t>
-        </is>
-      </c>
-      <c r="M87" t="inlineStr">
-        <is>
-          <t>114</t>
-        </is>
-      </c>
-      <c r="N87" t="inlineStr">
-        <is>
-          <t>2.4</t>
-        </is>
-      </c>
-      <c r="O87" t="inlineStr">
-        <is>
-          <t>240</t>
-        </is>
-      </c>
-      <c r="P87" t="inlineStr">
-        <is>
-          <t>320</t>
-        </is>
-      </c>
-      <c r="Q87" t="inlineStr">
-        <is>
-          <t>167</t>
-        </is>
+      <c r="J87" t="n">
+        <v>118</v>
+      </c>
+      <c r="K87" t="n">
+        <v>53</v>
+      </c>
+      <c r="L87" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="M87" t="n">
+        <v>114</v>
+      </c>
+      <c r="N87" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="O87" t="n">
+        <v>240</v>
+      </c>
+      <c r="P87" t="n">
+        <v>320</v>
+      </c>
+      <c r="Q87" t="n">
+        <v>167</v>
       </c>
       <c r="R87" t="inlineStr">
         <is>
@@ -29214,10 +28772,8 @@
         </is>
       </c>
       <c r="S87" t="inlineStr"/>
-      <c r="T87" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="T87" t="n">
+        <v>2</v>
       </c>
       <c r="U87" t="inlineStr"/>
       <c r="V87" t="inlineStr"/>
@@ -29608,6 +29164,712 @@
       <c r="DJ88" t="inlineStr"/>
       <c r="DK88" t="inlineStr"/>
     </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Tecno</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Tecno Spark 4</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr"/>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>https://www.gsmarena.com/tecno_spark_4-10695.php</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>2026-06-03 05:21 UTC</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>2019, September 25. Released 2019, September 25</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Discontinued</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>165.3</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>75.9</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>8.2</t>
+        </is>
+      </c>
+      <c r="M89" t="inlineStr"/>
+      <c r="N89" t="inlineStr">
+        <is>
+          <t>6.52</t>
+        </is>
+      </c>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>720</t>
+        </is>
+      </c>
+      <c r="P89" t="inlineStr">
+        <is>
+          <t>1600</t>
+        </is>
+      </c>
+      <c r="Q89" t="inlineStr">
+        <is>
+          <t>269</t>
+        </is>
+      </c>
+      <c r="R89" t="inlineStr">
+        <is>
+          <t>32GB</t>
+        </is>
+      </c>
+      <c r="S89" t="inlineStr">
+        <is>
+          <t>2GB | 3GB</t>
+        </is>
+      </c>
+      <c r="T89" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="U89" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="V89" t="inlineStr">
+        <is>
+          <t>4000</t>
+        </is>
+      </c>
+      <c r="W89" t="inlineStr"/>
+      <c r="X89" t="inlineStr"/>
+      <c r="Y89" t="inlineStr"/>
+      <c r="Z89" t="inlineStr"/>
+      <c r="AA89" t="inlineStr"/>
+      <c r="AB89" t="inlineStr"/>
+      <c r="AC89" t="inlineStr"/>
+      <c r="AD89" t="inlineStr"/>
+      <c r="AE89" t="inlineStr"/>
+      <c r="AF89" t="inlineStr"/>
+      <c r="AG89" t="inlineStr"/>
+      <c r="AH89" t="inlineStr"/>
+      <c r="AI89" t="inlineStr">
+        <is>
+          <t>Li-Ion 4000 mAh</t>
+        </is>
+      </c>
+      <c r="AJ89" t="inlineStr"/>
+      <c r="AK89" t="inlineStr">
+        <is>
+          <t>165.3 x 75.9 x 8.2 mm (6.51 x 2.99 x 0.32 in)</t>
+        </is>
+      </c>
+      <c r="AL89" t="inlineStr">
+        <is>
+          <t>Nano-SIM + Nano-SIM</t>
+        </is>
+      </c>
+      <c r="AM89" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AN89" t="inlineStr"/>
+      <c r="AO89" t="inlineStr">
+        <is>
+          <t>4.2, A2DP, LE</t>
+        </is>
+      </c>
+      <c r="AP89" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AQ89" t="inlineStr">
+        <is>
+          <t>GPS</t>
+        </is>
+      </c>
+      <c r="AR89" t="inlineStr">
+        <is>
+          <t>FM radio</t>
+        </is>
+      </c>
+      <c r="AS89" t="inlineStr">
+        <is>
+          <t>microUSB 2.0, OTG</t>
+        </is>
+      </c>
+      <c r="AT89" t="inlineStr">
+        <is>
+          <t>Wi-Fi 802.11 b/g/n</t>
+        </is>
+      </c>
+      <c r="AU89" t="inlineStr"/>
+      <c r="AV89" t="inlineStr"/>
+      <c r="AW89" t="inlineStr">
+        <is>
+          <t>720 x 1600 pixels, 20:9 ratio (~269 ppi density)</t>
+        </is>
+      </c>
+      <c r="AX89" t="inlineStr">
+        <is>
+          <t>6.52 inches, 102.6 cm 2 (~81.8% screen-to-body ratio)</t>
+        </is>
+      </c>
+      <c r="AY89" t="inlineStr">
+        <is>
+          <t>IPS LCD</t>
+        </is>
+      </c>
+      <c r="AZ89" t="inlineStr"/>
+      <c r="BA89" t="inlineStr"/>
+      <c r="BB89" t="inlineStr"/>
+      <c r="BC89" t="inlineStr"/>
+      <c r="BD89" t="inlineStr"/>
+      <c r="BE89" t="inlineStr"/>
+      <c r="BF89" t="inlineStr"/>
+      <c r="BG89" t="inlineStr"/>
+      <c r="BH89" t="inlineStr"/>
+      <c r="BI89" t="inlineStr"/>
+      <c r="BJ89" t="inlineStr"/>
+      <c r="BK89" t="inlineStr"/>
+      <c r="BL89" t="inlineStr">
+        <is>
+          <t>Fingerprint (rear-mounted), accelerometer, proximity</t>
+        </is>
+      </c>
+      <c r="BM89" t="inlineStr">
+        <is>
+          <t>2019, September 25. Released 2019, September 25</t>
+        </is>
+      </c>
+      <c r="BN89" t="inlineStr">
+        <is>
+          <t>Discontinued</t>
+        </is>
+      </c>
+      <c r="BO89" t="inlineStr"/>
+      <c r="BP89" t="inlineStr">
+        <is>
+          <t>Dual LED flash, HDR, panorama</t>
+        </is>
+      </c>
+      <c r="BQ89" t="inlineStr"/>
+      <c r="BR89" t="inlineStr">
+        <is>
+          <t>13 MP, AF Auxiliary lenses</t>
+        </is>
+      </c>
+      <c r="BS89" t="inlineStr">
+        <is>
+          <t>1080p@30fps</t>
+        </is>
+      </c>
+      <c r="BT89" t="inlineStr">
+        <is>
+          <t>eMMC 5.1</t>
+        </is>
+      </c>
+      <c r="BU89" t="inlineStr"/>
+      <c r="BV89" t="inlineStr">
+        <is>
+          <t>microSDXC (dedicated slot)</t>
+        </is>
+      </c>
+      <c r="BW89" t="inlineStr">
+        <is>
+          <t>32GB 2GB RAM, 32GB 3GB RAM</t>
+        </is>
+      </c>
+      <c r="BX89" t="inlineStr"/>
+      <c r="BY89" t="inlineStr">
+        <is>
+          <t>Royal Purple, Vacation Blue</t>
+        </is>
+      </c>
+      <c r="BZ89" t="inlineStr">
+        <is>
+          <t>KC8</t>
+        </is>
+      </c>
+      <c r="CA89" t="inlineStr"/>
+      <c r="CB89" t="inlineStr"/>
+      <c r="CC89" t="inlineStr"/>
+      <c r="CD89" t="inlineStr"/>
+      <c r="CE89" t="inlineStr"/>
+      <c r="CF89" t="inlineStr">
+        <is>
+          <t>GSM 850 / 900 / 1800 / 1900</t>
+        </is>
+      </c>
+      <c r="CG89" t="inlineStr">
+        <is>
+          <t>HSDPA 850 / 900 / 2100</t>
+        </is>
+      </c>
+      <c r="CH89" t="inlineStr">
+        <is>
+          <t>1, 3, 5, 8, 38, 40, 41</t>
+        </is>
+      </c>
+      <c r="CI89" t="inlineStr"/>
+      <c r="CJ89" t="inlineStr"/>
+      <c r="CK89" t="inlineStr"/>
+      <c r="CL89" t="inlineStr">
+        <is>
+          <t>HSPA 42.2/5.76 Mbps, LTE Cat4 150/50 Mbps</t>
+        </is>
+      </c>
+      <c r="CM89" t="inlineStr">
+        <is>
+          <t>GSM / HSPA / LTE</t>
+        </is>
+      </c>
+      <c r="CN89" t="inlineStr"/>
+      <c r="CO89" t="inlineStr">
+        <is>
+          <t>Quad-core 2.0 GHz</t>
+        </is>
+      </c>
+      <c r="CP89" t="inlineStr"/>
+      <c r="CQ89" t="inlineStr"/>
+      <c r="CR89" t="inlineStr">
+        <is>
+          <t>Android 9.0 (Pie), HIOS 5.5</t>
+        </is>
+      </c>
+      <c r="CS89" t="inlineStr"/>
+      <c r="CT89" t="inlineStr">
+        <is>
+          <t>8 MP</t>
+        </is>
+      </c>
+      <c r="CU89" t="inlineStr">
+        <is>
+          <t>1080p@30fps</t>
+        </is>
+      </c>
+      <c r="CV89" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="CW89" t="inlineStr"/>
+      <c r="CX89" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="CY89" t="inlineStr"/>
+      <c r="CZ89" t="inlineStr"/>
+      <c r="DA89" t="inlineStr"/>
+      <c r="DB89" t="inlineStr"/>
+      <c r="DC89" t="inlineStr"/>
+      <c r="DD89" t="inlineStr"/>
+      <c r="DE89" t="inlineStr">
+        <is>
+          <t>Glass front, plastic back, plastic frame</t>
+        </is>
+      </c>
+      <c r="DF89" t="inlineStr"/>
+      <c r="DG89" t="inlineStr"/>
+      <c r="DH89" t="inlineStr"/>
+      <c r="DI89" t="inlineStr"/>
+      <c r="DJ89" t="inlineStr"/>
+      <c r="DK89" t="inlineStr">
+        <is>
+          <t>LED flash</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Tecno</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Tecno Camon 12 Pro</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr"/>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>https://www.gsmarena.com/tecno_camon_12_pro-9865.php</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>2026-06-03 05:21 UTC</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>2019, September. Released 2019, September</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Discontinued</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>158.6</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>75.5</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>7.8</t>
+        </is>
+      </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>161</t>
+        </is>
+      </c>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t>6.35</t>
+        </is>
+      </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>720</t>
+        </is>
+      </c>
+      <c r="P90" t="inlineStr">
+        <is>
+          <t>1600</t>
+        </is>
+      </c>
+      <c r="Q90" t="inlineStr">
+        <is>
+          <t>276</t>
+        </is>
+      </c>
+      <c r="R90" t="inlineStr">
+        <is>
+          <t>64GB</t>
+        </is>
+      </c>
+      <c r="S90" t="inlineStr">
+        <is>
+          <t>6GB</t>
+        </is>
+      </c>
+      <c r="T90" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="U90" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="V90" t="inlineStr">
+        <is>
+          <t>3500</t>
+        </is>
+      </c>
+      <c r="W90" t="inlineStr"/>
+      <c r="X90" t="inlineStr"/>
+      <c r="Y90" t="inlineStr"/>
+      <c r="Z90" t="inlineStr"/>
+      <c r="AA90" t="inlineStr"/>
+      <c r="AB90" t="inlineStr"/>
+      <c r="AC90" t="inlineStr"/>
+      <c r="AD90" t="inlineStr"/>
+      <c r="AE90" t="inlineStr">
+        <is>
+          <t>About 10000 INR</t>
+        </is>
+      </c>
+      <c r="AF90" t="inlineStr"/>
+      <c r="AG90" t="inlineStr"/>
+      <c r="AH90" t="inlineStr"/>
+      <c r="AI90" t="inlineStr">
+        <is>
+          <t>3500 mAh, non-removable</t>
+        </is>
+      </c>
+      <c r="AJ90" t="inlineStr"/>
+      <c r="AK90" t="inlineStr">
+        <is>
+          <t>158.6 x 75.5 x 7.8 mm (6.24 x 2.97 x 0.31 in)</t>
+        </is>
+      </c>
+      <c r="AL90" t="inlineStr">
+        <is>
+          <t>Nano-SIM + Nano-SIM</t>
+        </is>
+      </c>
+      <c r="AM90" t="inlineStr">
+        <is>
+          <t>161 g (5.68 oz)</t>
+        </is>
+      </c>
+      <c r="AN90" t="inlineStr"/>
+      <c r="AO90" t="inlineStr">
+        <is>
+          <t>5.0, A2DP, LE</t>
+        </is>
+      </c>
+      <c r="AP90" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AQ90" t="inlineStr">
+        <is>
+          <t>GPS</t>
+        </is>
+      </c>
+      <c r="AR90" t="inlineStr">
+        <is>
+          <t>FM radio</t>
+        </is>
+      </c>
+      <c r="AS90" t="inlineStr">
+        <is>
+          <t>microUSB 2.0</t>
+        </is>
+      </c>
+      <c r="AT90" t="inlineStr">
+        <is>
+          <t>Wi-Fi 802.11 a/b/g/n</t>
+        </is>
+      </c>
+      <c r="AU90" t="inlineStr"/>
+      <c r="AV90" t="inlineStr"/>
+      <c r="AW90" t="inlineStr">
+        <is>
+          <t>720 x 1600 pixels, 20:9 ratio (~276 ppi density)</t>
+        </is>
+      </c>
+      <c r="AX90" t="inlineStr">
+        <is>
+          <t>6.35 inches, 97.4 cm 2 (~81.3% screen-to-body ratio)</t>
+        </is>
+      </c>
+      <c r="AY90" t="inlineStr">
+        <is>
+          <t>AMOLED</t>
+        </is>
+      </c>
+      <c r="AZ90" t="inlineStr"/>
+      <c r="BA90" t="inlineStr"/>
+      <c r="BB90" t="inlineStr"/>
+      <c r="BC90" t="inlineStr"/>
+      <c r="BD90" t="inlineStr"/>
+      <c r="BE90" t="inlineStr"/>
+      <c r="BF90" t="inlineStr"/>
+      <c r="BG90" t="inlineStr"/>
+      <c r="BH90" t="inlineStr"/>
+      <c r="BI90" t="inlineStr"/>
+      <c r="BJ90" t="inlineStr"/>
+      <c r="BK90" t="inlineStr"/>
+      <c r="BL90" t="inlineStr">
+        <is>
+          <t>Fingerprint (under display, optical), accelerometer, proximity</t>
+        </is>
+      </c>
+      <c r="BM90" t="inlineStr">
+        <is>
+          <t>2019, September. Released 2019, September</t>
+        </is>
+      </c>
+      <c r="BN90" t="inlineStr">
+        <is>
+          <t>Discontinued</t>
+        </is>
+      </c>
+      <c r="BO90" t="inlineStr"/>
+      <c r="BP90" t="inlineStr">
+        <is>
+          <t>Quad-LED flash, panorama, HDR</t>
+        </is>
+      </c>
+      <c r="BQ90" t="inlineStr"/>
+      <c r="BR90" t="inlineStr">
+        <is>
+          <t>16 MP, PDAF 8 MP Auxiliary lens</t>
+        </is>
+      </c>
+      <c r="BS90" t="inlineStr">
+        <is>
+          <t>1080p@30fps</t>
+        </is>
+      </c>
+      <c r="BT90" t="inlineStr">
+        <is>
+          <t>eMMC 5.1</t>
+        </is>
+      </c>
+      <c r="BU90" t="inlineStr"/>
+      <c r="BV90" t="inlineStr">
+        <is>
+          <t>microSDXC (dedicated slot)</t>
+        </is>
+      </c>
+      <c r="BW90" t="inlineStr">
+        <is>
+          <t>64GB 6GB RAM</t>
+        </is>
+      </c>
+      <c r="BX90" t="inlineStr"/>
+      <c r="BY90" t="inlineStr">
+        <is>
+          <t>Dawn Blue</t>
+        </is>
+      </c>
+      <c r="BZ90" t="inlineStr"/>
+      <c r="CA90" t="inlineStr">
+        <is>
+          <t>About 10000 INR</t>
+        </is>
+      </c>
+      <c r="CB90" t="inlineStr"/>
+      <c r="CC90" t="inlineStr"/>
+      <c r="CD90" t="inlineStr"/>
+      <c r="CE90" t="inlineStr"/>
+      <c r="CF90" t="inlineStr">
+        <is>
+          <t>GSM 850 / 900 / 1800 / 1900</t>
+        </is>
+      </c>
+      <c r="CG90" t="inlineStr">
+        <is>
+          <t>HSDPA 850 / 900 / 1700(AWS) / 1900 / 2100</t>
+        </is>
+      </c>
+      <c r="CH90" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 7, 8, 20, 28</t>
+        </is>
+      </c>
+      <c r="CI90" t="inlineStr"/>
+      <c r="CJ90" t="inlineStr"/>
+      <c r="CK90" t="inlineStr"/>
+      <c r="CL90" t="inlineStr">
+        <is>
+          <t>HSPA 42.2/5.76 Mbps, LTE Cat4 150/50 Mbps</t>
+        </is>
+      </c>
+      <c r="CM90" t="inlineStr">
+        <is>
+          <t>GSM / HSPA / LTE</t>
+        </is>
+      </c>
+      <c r="CN90" t="inlineStr"/>
+      <c r="CO90" t="inlineStr">
+        <is>
+          <t>Octa-core 2.0 GHz Cortex-A53</t>
+        </is>
+      </c>
+      <c r="CP90" t="inlineStr">
+        <is>
+          <t>Mediatek MT6762 Helio P22 (12 nm)</t>
+        </is>
+      </c>
+      <c r="CQ90" t="inlineStr">
+        <is>
+          <t>PowerVR GE8320</t>
+        </is>
+      </c>
+      <c r="CR90" t="inlineStr">
+        <is>
+          <t>Android 9.0 (Pie), HIOS 5.5</t>
+        </is>
+      </c>
+      <c r="CS90" t="inlineStr"/>
+      <c r="CT90" t="inlineStr">
+        <is>
+          <t>32 MP, f/2.0, 26mm (wide), 1/2.8", 0.8µm</t>
+        </is>
+      </c>
+      <c r="CU90" t="inlineStr">
+        <is>
+          <t>1080p@30fps</t>
+        </is>
+      </c>
+      <c r="CV90" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="CW90" t="inlineStr"/>
+      <c r="CX90" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="CY90" t="inlineStr"/>
+      <c r="CZ90" t="inlineStr"/>
+      <c r="DA90" t="inlineStr"/>
+      <c r="DB90" t="inlineStr"/>
+      <c r="DC90" t="inlineStr"/>
+      <c r="DD90" t="inlineStr"/>
+      <c r="DE90" t="inlineStr">
+        <is>
+          <t>Glass front, plastic back, plastic frame</t>
+        </is>
+      </c>
+      <c r="DF90" t="inlineStr"/>
+      <c r="DG90" t="inlineStr"/>
+      <c r="DH90" t="inlineStr"/>
+      <c r="DI90" t="inlineStr"/>
+      <c r="DJ90" t="inlineStr"/>
+      <c r="DK90" t="inlineStr">
+        <is>
+          <t>LED flash, HDR</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
New devices scraped 2026-06-03 14:34 UTC
</commit_message>
<xml_diff>
--- a/gsmarena_new_2026-06-03.xlsx
+++ b/gsmarena_new_2026-06-03.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY3"/>
+  <dimension ref="A1:BE6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -672,6 +672,36 @@
           <t>Misc_Models</t>
         </is>
       </c>
+      <c r="AZ1" t="inlineStr">
+        <is>
+          <t>Memory</t>
+        </is>
+      </c>
+      <c r="BA1" t="inlineStr">
+        <is>
+          <t>Main Camera_Single</t>
+        </is>
+      </c>
+      <c r="BB1" t="inlineStr">
+        <is>
+          <t>Network</t>
+        </is>
+      </c>
+      <c r="BC1" t="inlineStr">
+        <is>
+          <t>Network_2</t>
+        </is>
+      </c>
+      <c r="BD1" t="inlineStr">
+        <is>
+          <t>Main Camera_Penta</t>
+        </is>
+      </c>
+      <c r="BE1" t="inlineStr">
+        <is>
+          <t>Selfie camera_Features</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -694,10 +724,8 @@
           <t>2026-06-03 14:07 UTC</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
+      <c r="E2" t="n">
+        <v>2025</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -909,6 +937,12 @@
       <c r="AW2" t="inlineStr"/>
       <c r="AX2" t="inlineStr"/>
       <c r="AY2" t="inlineStr"/>
+      <c r="AZ2" t="inlineStr"/>
+      <c r="BA2" t="inlineStr"/>
+      <c r="BB2" t="inlineStr"/>
+      <c r="BC2" t="inlineStr"/>
+      <c r="BD2" t="inlineStr"/>
+      <c r="BE2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -931,10 +965,8 @@
           <t>2026-06-03 14:07 UTC</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
+      <c r="E3" t="n">
+        <v>2025</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1146,6 +1178,761 @@
           <t>ZL.H01SI.002</t>
         </is>
       </c>
+      <c r="AZ3" t="inlineStr"/>
+      <c r="BA3" t="inlineStr"/>
+      <c r="BB3" t="inlineStr"/>
+      <c r="BC3" t="inlineStr"/>
+      <c r="BD3" t="inlineStr"/>
+      <c r="BE3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Ulefone</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Ulefone Tab A7</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://www.gsmarena.com/ulefone_tab_a7-10994.php</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-06-03 14:33 UTC</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2021, May 27</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Available. Released 2021, May 27</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>GSM / HSPA / LTE</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>GSM 850 / 900 / 1800 / 1900</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>HSDPA 850 / 900 / 1900 / 2100</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 5, 7, 8, 20</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>HSPA 21.1/5.76 Mbps, LTE Cat4 150/50 Mbps</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>2021, May 27</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Available. Released 2021, May 27</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>243.6 x 162.4 x 7.9 mm (9.59 x 6.39 x 0.31 in)</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>566 g (1.25 lb)</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Nano-SIM + Nano-SIM</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>IPS LCD</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>10.1 inches, 295.8 cm 2 (~74.8% screen-to-body ratio)</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>1200 x 1920 pixels, 16:10 ratio (~224 ppi density)</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>Android 11</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>Unisoc SC9863A (28 nm)</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>Octa-core (4x1.6 GHz Cortex-A55 &amp; 4x1.2 GHz Cortex-A55)</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>IMG8322</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>microSDXC (uses shared SIM slot)</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>64GB 4GB RAM</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr"/>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>LED flash, HDR, panorama</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>4K@30fps, 1080p@30fps</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>5 MP</t>
+        </is>
+      </c>
+      <c r="AG4" t="inlineStr"/>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AJ4" t="inlineStr">
+        <is>
+          <t>Wi-Fi 802.11 a/b/g/n/ac, dual-band</t>
+        </is>
+      </c>
+      <c r="AK4" t="inlineStr">
+        <is>
+          <t>5.0, A2DP, LE</t>
+        </is>
+      </c>
+      <c r="AL4" t="inlineStr">
+        <is>
+          <t>GPS, GLONASS, BDS</t>
+        </is>
+      </c>
+      <c r="AM4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AN4" t="inlineStr">
+        <is>
+          <t>FM radio, RDS, recording</t>
+        </is>
+      </c>
+      <c r="AO4" t="inlineStr">
+        <is>
+          <t>USB Type-C 2.0, OTG</t>
+        </is>
+      </c>
+      <c r="AP4" t="inlineStr">
+        <is>
+          <t>Accelerometer, proximity</t>
+        </is>
+      </c>
+      <c r="AQ4" t="inlineStr">
+        <is>
+          <t>Li-Po 7680 mAh</t>
+        </is>
+      </c>
+      <c r="AR4" t="inlineStr">
+        <is>
+          <t>10W wired</t>
+        </is>
+      </c>
+      <c r="AS4" t="inlineStr">
+        <is>
+          <t>Space Gray</t>
+        </is>
+      </c>
+      <c r="AT4" t="inlineStr">
+        <is>
+          <t>About 130 EUR</t>
+        </is>
+      </c>
+      <c r="AU4" t="inlineStr"/>
+      <c r="AV4" t="inlineStr"/>
+      <c r="AW4" t="inlineStr"/>
+      <c r="AX4" t="inlineStr"/>
+      <c r="AY4" t="inlineStr"/>
+      <c r="AZ4" t="inlineStr">
+        <is>
+          <t>eMMC 5.1</t>
+        </is>
+      </c>
+      <c r="BA4" t="inlineStr">
+        <is>
+          <t>13 MP</t>
+        </is>
+      </c>
+      <c r="BB4" t="inlineStr"/>
+      <c r="BC4" t="inlineStr"/>
+      <c r="BD4" t="inlineStr"/>
+      <c r="BE4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Ulefone</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Ulefone Armor 11T 5G</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://www.gsmarena.com/ulefone_armor_11t_5g-10974.php</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2026-06-03 14:33 UTC</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2021, May 29</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Available. Released 2021, June 07</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>GSM / CDMA / HSPA / EVDO / LTE / 5G</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>GSM 850 / 900 / 1800 / 1900</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>HSDPA 850 / 900 / 1700(AWS) / 1900 / 2100</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 7, 8, 12, 13, 17, 18, 19, 20, 25, 26, 28, 34, 38, 39, 40, 41, 66</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>1, 3, 5, 8, 20, 28, 38, 41, 77, 78, 79 SA/NSA</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>HSPA, LTE, 5G</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>2021, May 29</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Available. Released 2021, June 07</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>163.8 x 81.6 x 14.2 mm (6.45 x 3.21 x 0.56 in)</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>293 g (10.34 oz)</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Nano-SIM + Nano-SIM</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>IP68/IP69K dust tight and water resistant (high pressure water jets; immersible up to 1.5m for 30 min) Drop resistant up to 1.2m MIL-STD-810G compliant</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>IPS LCD</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>6.1 inches, 91.3 cm 2 (~68.3% screen-to-body ratio)</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>720 x 1560 pixels, 19.5:9 ratio (~282 ppi density)</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>Android 11</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>Mediatek Dimensity 800 (7 nm)</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>Octa-core (4x2.0 GHz Cortex-A76 &amp; 4x2.0 GHz Cortex-A55)</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>Mali-G57 MP4</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>256GB 8GB RAM</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr"/>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>Dual-LED dual-tone flash, HDR, panorama</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>4K@30fps, 1080p@30fps</t>
+        </is>
+      </c>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t>16 MP, f/2.0</t>
+        </is>
+      </c>
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t>1080p@30fps</t>
+        </is>
+      </c>
+      <c r="AH5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AI5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AJ5" t="inlineStr">
+        <is>
+          <t>Wi-Fi 802.11 a/b/g/n/ac, Wi-Fi Direct</t>
+        </is>
+      </c>
+      <c r="AK5" t="inlineStr">
+        <is>
+          <t>5.0, A2DP, LE</t>
+        </is>
+      </c>
+      <c r="AL5" t="inlineStr">
+        <is>
+          <t>GPS, GLONASS, GALILEO, BDS</t>
+        </is>
+      </c>
+      <c r="AM5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AN5" t="inlineStr">
+        <is>
+          <t>FM radio, RDS, recording</t>
+        </is>
+      </c>
+      <c r="AO5" t="inlineStr">
+        <is>
+          <t>USB Type-C 2.0, OTG</t>
+        </is>
+      </c>
+      <c r="AP5" t="inlineStr">
+        <is>
+          <t>Fingerprint (side-mounted), accelerometer, gyro, proximity, compass, baroceptor</t>
+        </is>
+      </c>
+      <c r="AQ5" t="inlineStr">
+        <is>
+          <t>Li-Po 5200 mAh</t>
+        </is>
+      </c>
+      <c r="AR5" t="inlineStr">
+        <is>
+          <t>18W wired 10W wireless</t>
+        </is>
+      </c>
+      <c r="AS5" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="AT5" t="inlineStr">
+        <is>
+          <t>About 590 EUR</t>
+        </is>
+      </c>
+      <c r="AU5" t="inlineStr">
+        <is>
+          <t>Front glass, aluminum back with rubber, aluminum frame</t>
+        </is>
+      </c>
+      <c r="AV5" t="inlineStr">
+        <is>
+          <t>Oleophobic coating</t>
+        </is>
+      </c>
+      <c r="AW5" t="inlineStr"/>
+      <c r="AX5" t="inlineStr"/>
+      <c r="AY5" t="inlineStr"/>
+      <c r="AZ5" t="inlineStr">
+        <is>
+          <t>UFS 2.1</t>
+        </is>
+      </c>
+      <c r="BA5" t="inlineStr"/>
+      <c r="BB5" t="inlineStr">
+        <is>
+          <t>CDMA 800 / 1900 &amp; TD-SCDMA</t>
+        </is>
+      </c>
+      <c r="BC5" t="inlineStr">
+        <is>
+          <t>CDMA2000 1xEV-DO</t>
+        </is>
+      </c>
+      <c r="BD5" t="inlineStr">
+        <is>
+          <t>48 MP, f/1.8, 26mm (wide), 1/2.0", 0.8µm, PDAF FLIR thermal camera (Lepton module) 5 MP 2 MP (macro) Auxiliary lens</t>
+        </is>
+      </c>
+      <c r="BE5" t="inlineStr">
+        <is>
+          <t>HDR, panorama</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Ulefone</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Ulefone Armor 8 Pro</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://www.gsmarena.com/ulefone_armor_8_pro-10898.php</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026-06-03 14:33 UTC</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2021, April 28</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Available. Released 2021, April 28</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>GSM / HSPA / LTE</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>GSM 850 / 900 / 1800 / 1900</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>HSDPA 850 / 900 / 1700(AWS) / 1900 / 2100</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 7, 8, 12, 13, 17, 18, 19, 20, 25, 26, 28, 66</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>HSPA 42.2/11.5 Mbps, LTE Cat7 300/150 Mbps</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>2021, April 28</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Available. Released 2021, April 28</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>166 x 81.8 x 15 mm (6.54 x 3.22 x 0.59 in)</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>282 g (9.95 oz)</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Nano-SIM + Nano-SIM</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>IP68 dust tight and water resistant (immersible up to 1.5m for 30 min) Drop resistant up to 1.2m MIL-STD-810G compliant</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>IPS LCD</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>6.1 inches, 91.3 cm 2 (~67.3% screen-to-body ratio)</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>720 x 1560 pixels, 19.5:9 ratio (~282 ppi density)</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>Android 11</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>Mediatek MT6771 Helio P60 (12 nm)</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>Octa-core (4x2.0 GHz Cortex-A73 &amp; 4x2.0 GHz Cortex-A53)</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>Mali-G72 MP3</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>microSDXC (uses shared SIM slot)</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>128GB 6GB RAM, 128GB 8GB RAM</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>16 MP, f/2.2, (wide), PDAF 5 MP (macro) Auxiliary lens</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>LED flash, Panorama, HDR</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>1080p@30fps</t>
+        </is>
+      </c>
+      <c r="AF6" t="inlineStr">
+        <is>
+          <t>8 MP, f/2.2</t>
+        </is>
+      </c>
+      <c r="AG6" t="inlineStr">
+        <is>
+          <t>1080p@30fps</t>
+        </is>
+      </c>
+      <c r="AH6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AI6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AJ6" t="inlineStr">
+        <is>
+          <t>Wi-Fi 802.11 a/b/g/n/ac, Wi-Fi Direct</t>
+        </is>
+      </c>
+      <c r="AK6" t="inlineStr">
+        <is>
+          <t>4.2, A2DP, LE</t>
+        </is>
+      </c>
+      <c r="AL6" t="inlineStr">
+        <is>
+          <t>GPS, GLONASS, GALILEO, BDS</t>
+        </is>
+      </c>
+      <c r="AM6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AN6" t="inlineStr">
+        <is>
+          <t>FM radio, RDS, recording</t>
+        </is>
+      </c>
+      <c r="AO6" t="inlineStr">
+        <is>
+          <t>USB Type-C 2.0, OTG</t>
+        </is>
+      </c>
+      <c r="AP6" t="inlineStr">
+        <is>
+          <t>Fingerprint (side-mounted), accelerometer, gyro, proximity, compass</t>
+        </is>
+      </c>
+      <c r="AQ6" t="inlineStr">
+        <is>
+          <t>Li-Po 5580 mAh</t>
+        </is>
+      </c>
+      <c r="AR6" t="inlineStr">
+        <is>
+          <t>15W wired</t>
+        </is>
+      </c>
+      <c r="AS6" t="inlineStr">
+        <is>
+          <t>Black, Orange, Red</t>
+        </is>
+      </c>
+      <c r="AT6" t="inlineStr">
+        <is>
+          <t>About 190 EUR</t>
+        </is>
+      </c>
+      <c r="AU6" t="inlineStr">
+        <is>
+          <t>Front glass, aluminum back with rubber, aluminum frame</t>
+        </is>
+      </c>
+      <c r="AV6" t="inlineStr">
+        <is>
+          <t>Scratch-resistant glass, oleophobic coating</t>
+        </is>
+      </c>
+      <c r="AW6" t="inlineStr"/>
+      <c r="AX6" t="inlineStr"/>
+      <c r="AY6" t="inlineStr"/>
+      <c r="AZ6" t="inlineStr"/>
+      <c r="BA6" t="inlineStr"/>
+      <c r="BB6" t="inlineStr"/>
+      <c r="BC6" t="inlineStr"/>
+      <c r="BD6" t="inlineStr"/>
+      <c r="BE6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>